<commit_message>
Stabilize live data render and bubble movement lines
</commit_message>
<xml_diff>
--- a/data/portfolio-data.xlsx
+++ b/data/portfolio-data.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Data" sheetId="1" r:id="Rdcce941969ae4d65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R7a5ee3a0a8e64fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Data" sheetId="1" r:id="Ref24b1e7997548cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R2832b5cf3f2d44e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -970,7 +970,7 @@
         <x:v>122000</x:v>
       </x:c>
       <x:c r="F7" s="33" t="n">
-        <x:v>105000</x:v>
+        <x:v>107000</x:v>
       </x:c>
       <x:c r="G7" s="34" t="n">
         <x:v>0.91</x:v>
@@ -980,11 +980,11 @@
       </x:c>
       <x:c r="I7" s="22" t="n">
         <x:f>IF(OR($G7="",$F7=""),"",ROUND($G7*1000000/$F7,2))</x:f>
-        <x:v>8.67</x:v>
+        <x:v>8.5</x:v>
       </x:c>
       <x:c r="J7" s="22" t="n">
         <x:f>IF(OR($H7="",$F7=""),"",ROUND($H7*1000000/$F7,1))</x:f>
-        <x:v>31.2</x:v>
+        <x:v>30.7</x:v>
       </x:c>
       <x:c r="K7" s="35" t="n">
         <x:v>8.3</x:v>
@@ -994,7 +994,7 @@
       </x:c>
       <x:c r="M7" s="24" t="n">
         <x:f>IF(OR(I7="",J7="",K7="",L7=""),"",ROUND(MIN(100,MAX(0,MIN(35,MAX(0,(I7-8)/6*35))+MIN(35,MAX(0,(J7-20)/16*35))+MIN(30,MAX(0,(((I7/K7)-1)+((J7/L7)-1))/0.25*30)))),0))</x:f>
-        <x:v>38</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="N7" s="25" t="str">
         <x:f>IF($M7="","",IF($M7&gt;=75,"hot",IF($M7&gt;=55,"warn","good")))</x:f>

</xml_diff>

<commit_message>
Add password protection to Excel workbook
</commit_message>
<xml_diff>
--- a/data/portfolio-data.xlsx
+++ b/data/portfolio-data.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Data" sheetId="1" r:id="Ref24b1e7997548cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R2832b5cf3f2d44e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Data" sheetId="1" r:id="Ra26f274bfd804ed4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="Ra427ef6e56e64715"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -327,7 +327,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1"/>
+  <x:sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="0" selectUnlockedCells="1" password="DF4A"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16.670000076293945" hidden="0" customWidth="1"/>

</xml_diff>